<commit_message>
add info tags to xlsx
</commit_message>
<xml_diff>
--- a/api/templates/results_10a_10b_covid_ntp_use/en.xlsx
+++ b/api/templates/results_10a_10b_covid_ntp_use/en.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu-20.04\home\maiki\.oh-my-zsh\aspect\api\templates\results_10a_10b_covid_ntp_use\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBD7FC9C-1B69-45C4-A2EF-498923B957EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5AFEC5A-AF90-4F0F-B58C-58570DDA85B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12552" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="January" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="113">
   <si>
     <t>Sl No.</t>
   </si>
@@ -221,9 +221,6 @@
     <t>&lt;presumptiveUnknown&gt;</t>
   </si>
   <si>
-    <t>&lt;presumptiveAll&gt;</t>
-  </si>
-  <si>
     <t>&lt;col3&gt;</t>
   </si>
   <si>
@@ -300,6 +297,102 @@
   </si>
   <si>
     <t>&lt;sumMe&gt;</t>
+  </si>
+  <si>
+    <t>c6</t>
+  </si>
+  <si>
+    <t>c7</t>
+  </si>
+  <si>
+    <t>c8</t>
+  </si>
+  <si>
+    <t>nombres aca</t>
+  </si>
+  <si>
+    <t>b26-26-32</t>
+  </si>
+  <si>
+    <t>c26-29-32</t>
+  </si>
+  <si>
+    <t>f5+g5</t>
+  </si>
+  <si>
+    <t>e26-29-32</t>
+  </si>
+  <si>
+    <t>f26-29-32</t>
+  </si>
+  <si>
+    <t>g26-29-32</t>
+  </si>
+  <si>
+    <t>h26-29-32</t>
+  </si>
+  <si>
+    <t>i26-29-32</t>
+  </si>
+  <si>
+    <t>j26-29-32</t>
+  </si>
+  <si>
+    <t>k26-29-32</t>
+  </si>
+  <si>
+    <t>l26-29-32</t>
+  </si>
+  <si>
+    <t>026-29-32</t>
+  </si>
+  <si>
+    <t>o27-30-33</t>
+  </si>
+  <si>
+    <t>o28-31-34</t>
+  </si>
+  <si>
+    <t>r26-29-32</t>
+  </si>
+  <si>
+    <t>R27-30-33</t>
+  </si>
+  <si>
+    <t>r28-31-34</t>
+  </si>
+  <si>
+    <t>m40-p40-s40</t>
+  </si>
+  <si>
+    <t>m41-p41-s41</t>
+  </si>
+  <si>
+    <t>m42-p42-s42</t>
+  </si>
+  <si>
+    <t>n40-q40-t40</t>
+  </si>
+  <si>
+    <t>n41-q41-t41</t>
+  </si>
+  <si>
+    <t>n42-q42-t42</t>
+  </si>
+  <si>
+    <t>o41-r40-u40</t>
+  </si>
+  <si>
+    <t>o41-r41-u41</t>
+  </si>
+  <si>
+    <t>E26+F26+G26+H26+I26+J26+K26+L26+O26+O27+O28+R26+R27+R28+S26</t>
+  </si>
+  <si>
+    <t>O26+O27+O28+R26+R27+R28+S26</t>
+  </si>
+  <si>
+    <t>i5+j5+k5+l5+m5+n5+o5+p5+q5+r5+s5+t5+u5+v5</t>
   </si>
 </sst>
 </file>
@@ -676,10 +769,58 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
@@ -688,7 +829,67 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
@@ -709,114 +910,6 @@
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
@@ -1173,7 +1266,7 @@
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="A1:BI13"/>
+  <dimension ref="A1:BI18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.6640625" customWidth="1"/>
@@ -1184,7 +1277,19 @@
     <col min="7" max="7" width="16.88671875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.21875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.109375" customWidth="1"/>
-    <col min="10" max="31" width="9.109375" customWidth="1"/>
+    <col min="10" max="16" width="9.109375" customWidth="1"/>
+    <col min="17" max="17" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.109375" customWidth="1"/>
+    <col min="21" max="21" width="10.6640625" customWidth="1"/>
+    <col min="22" max="22" width="10.77734375" customWidth="1"/>
+    <col min="23" max="23" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="8.44140625" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="10.109375" customWidth="1"/>
     <col min="33" max="33" width="9.109375" customWidth="1"/>
     <col min="34" max="34" width="10.109375" customWidth="1"/>
@@ -1205,264 +1310,264 @@
       </c>
     </row>
     <row r="2" spans="1:61" s="1" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="14"/>
-      <c r="F2" s="17" t="s">
+      <c r="E2" s="41"/>
+      <c r="F2" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="39" t="s">
+      <c r="G2" s="37"/>
+      <c r="H2" s="37"/>
+      <c r="I2" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="39"/>
-      <c r="K2" s="39"/>
-      <c r="L2" s="39"/>
-      <c r="M2" s="39"/>
-      <c r="N2" s="39"/>
-      <c r="O2" s="39"/>
-      <c r="P2" s="39"/>
-      <c r="Q2" s="39"/>
-      <c r="R2" s="39"/>
-      <c r="S2" s="39"/>
-      <c r="T2" s="39"/>
-      <c r="U2" s="39"/>
-      <c r="V2" s="39"/>
-      <c r="W2" s="39"/>
-      <c r="X2" s="39"/>
-      <c r="Y2" s="39"/>
-      <c r="Z2" s="39"/>
-      <c r="AA2" s="39"/>
-      <c r="AB2" s="39"/>
-      <c r="AC2" s="39"/>
-      <c r="AD2" s="39"/>
-      <c r="AE2" s="39"/>
-      <c r="AF2" s="39"/>
-      <c r="AG2" s="39"/>
-      <c r="AH2" s="40" t="s">
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="13"/>
+      <c r="P2" s="13"/>
+      <c r="Q2" s="13"/>
+      <c r="R2" s="13"/>
+      <c r="S2" s="13"/>
+      <c r="T2" s="13"/>
+      <c r="U2" s="13"/>
+      <c r="V2" s="13"/>
+      <c r="W2" s="13"/>
+      <c r="X2" s="13"/>
+      <c r="Y2" s="13"/>
+      <c r="Z2" s="13"/>
+      <c r="AA2" s="13"/>
+      <c r="AB2" s="13"/>
+      <c r="AC2" s="13"/>
+      <c r="AD2" s="13"/>
+      <c r="AE2" s="13"/>
+      <c r="AF2" s="13"/>
+      <c r="AG2" s="13"/>
+      <c r="AH2" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="AI2" s="40"/>
-      <c r="AJ2" s="40"/>
-      <c r="AK2" s="40"/>
-      <c r="AL2" s="8" t="s">
+      <c r="AI2" s="14"/>
+      <c r="AJ2" s="14"/>
+      <c r="AK2" s="14"/>
+      <c r="AL2" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="AM2" s="8" t="s">
+      <c r="AM2" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="AN2" s="8" t="s">
+      <c r="AN2" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="AO2" s="9" t="s">
+      <c r="AO2" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="AP2" s="10"/>
-      <c r="AQ2" s="10"/>
-      <c r="AR2" s="30" t="s">
+      <c r="AP2" s="22"/>
+      <c r="AQ2" s="22"/>
+      <c r="AR2" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="AS2" s="9" t="s">
+      <c r="AS2" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="AT2" s="10"/>
-      <c r="AU2" s="10"/>
-      <c r="AV2" s="30" t="s">
+      <c r="AT2" s="22"/>
+      <c r="AU2" s="22"/>
+      <c r="AV2" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="AW2" s="9" t="s">
+      <c r="AW2" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="AX2" s="10"/>
-      <c r="AY2" s="10"/>
-      <c r="AZ2" s="30" t="s">
+      <c r="AX2" s="22"/>
+      <c r="AY2" s="22"/>
+      <c r="AZ2" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="BA2" s="9" t="s">
+      <c r="BA2" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="BB2" s="10"/>
-      <c r="BC2" s="33"/>
-      <c r="BD2" s="9" t="s">
+      <c r="BB2" s="22"/>
+      <c r="BC2" s="36"/>
+      <c r="BD2" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="BE2" s="10"/>
-      <c r="BF2" s="10"/>
-      <c r="BG2" s="21" t="s">
+      <c r="BE2" s="22"/>
+      <c r="BF2" s="22"/>
+      <c r="BG2" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="BH2" s="24" t="s">
+      <c r="BH2" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="BI2" s="25" t="s">
+      <c r="BI2" s="27" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:61" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="12"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="26" t="s">
+      <c r="A3" s="39"/>
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="28" t="s">
+      <c r="G3" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="29" t="s">
+      <c r="H3" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="11" t="s">
+      <c r="I3" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="J3" s="11" t="s">
+      <c r="J3" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="K3" s="11" t="s">
+      <c r="K3" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="L3" s="11" t="s">
+      <c r="L3" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="M3" s="11" t="s">
+      <c r="M3" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="N3" s="11" t="s">
+      <c r="N3" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="O3" s="11" t="s">
+      <c r="O3" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="P3" s="11" t="s">
+      <c r="P3" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="Q3" s="11" t="s">
+      <c r="Q3" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="R3" s="11"/>
-      <c r="S3" s="11"/>
-      <c r="T3" s="11" t="s">
+      <c r="R3" s="32"/>
+      <c r="S3" s="32"/>
+      <c r="T3" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="U3" s="11"/>
-      <c r="V3" s="11"/>
-      <c r="W3" s="20" t="s">
+      <c r="U3" s="32"/>
+      <c r="V3" s="32"/>
+      <c r="W3" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="X3" s="20"/>
-      <c r="Y3" s="20"/>
-      <c r="Z3" s="20" t="s">
+      <c r="X3" s="38"/>
+      <c r="Y3" s="38"/>
+      <c r="Z3" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="AA3" s="20"/>
-      <c r="AB3" s="20"/>
-      <c r="AC3" s="20" t="s">
+      <c r="AA3" s="38"/>
+      <c r="AB3" s="38"/>
+      <c r="AC3" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="AD3" s="20"/>
-      <c r="AE3" s="20"/>
-      <c r="AF3" s="42" t="s">
+      <c r="AD3" s="38"/>
+      <c r="AE3" s="38"/>
+      <c r="AF3" s="17" t="s">
         <v>37</v>
       </c>
       <c r="AG3" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="AH3" s="18" t="s">
+      <c r="AH3" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="AI3" s="18" t="s">
+      <c r="AI3" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="AJ3" s="18" t="s">
+      <c r="AJ3" s="20" t="s">
         <v>38</v>
       </c>
       <c r="AK3" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="AL3" s="8"/>
-      <c r="AM3" s="8"/>
-      <c r="AN3" s="8"/>
-      <c r="AO3" s="34" t="s">
+      <c r="AL3" s="15"/>
+      <c r="AM3" s="15"/>
+      <c r="AN3" s="15"/>
+      <c r="AO3" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="AP3" s="34" t="s">
+      <c r="AP3" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="AQ3" s="36" t="s">
+      <c r="AQ3" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="AR3" s="31"/>
-      <c r="AS3" s="34" t="s">
+      <c r="AR3" s="34"/>
+      <c r="AS3" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="AT3" s="41" t="s">
+      <c r="AT3" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="AU3" s="36" t="s">
+      <c r="AU3" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="AV3" s="31"/>
-      <c r="AW3" s="34" t="s">
+      <c r="AV3" s="34"/>
+      <c r="AW3" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="AX3" s="35" t="s">
+      <c r="AX3" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="AY3" s="36" t="s">
+      <c r="AY3" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="AZ3" s="31"/>
-      <c r="BA3" s="37" t="s">
+      <c r="AZ3" s="34"/>
+      <c r="BA3" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="BB3" s="37" t="s">
+      <c r="BB3" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="BC3" s="37" t="s">
+      <c r="BC3" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="BD3" s="37" t="s">
+      <c r="BD3" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="BE3" s="37" t="s">
+      <c r="BE3" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="BF3" s="37" t="s">
+      <c r="BF3" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="BG3" s="22"/>
-      <c r="BH3" s="24"/>
-      <c r="BI3" s="25"/>
+      <c r="BG3" s="24"/>
+      <c r="BH3" s="26"/>
+      <c r="BI3" s="27"/>
     </row>
     <row r="4" spans="1:61" s="1" customFormat="1" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="12"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="29"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
-      <c r="L4" s="11"/>
-      <c r="M4" s="11"/>
-      <c r="N4" s="11"/>
-      <c r="O4" s="11"/>
-      <c r="P4" s="11"/>
+      <c r="A4" s="39"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="32"/>
+      <c r="J4" s="32"/>
+      <c r="K4" s="32"/>
+      <c r="L4" s="32"/>
+      <c r="M4" s="32"/>
+      <c r="N4" s="32"/>
+      <c r="O4" s="32"/>
+      <c r="P4" s="32"/>
       <c r="Q4" s="2" t="s">
         <v>45</v>
       </c>
@@ -1508,36 +1613,36 @@
       <c r="AE4" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AF4" s="43"/>
+      <c r="AF4" s="18"/>
       <c r="AG4" s="19"/>
-      <c r="AH4" s="18"/>
-      <c r="AI4" s="18"/>
-      <c r="AJ4" s="18"/>
+      <c r="AH4" s="20"/>
+      <c r="AI4" s="20"/>
+      <c r="AJ4" s="20"/>
       <c r="AK4" s="19"/>
-      <c r="AL4" s="8"/>
-      <c r="AM4" s="8"/>
-      <c r="AN4" s="8"/>
-      <c r="AO4" s="34"/>
-      <c r="AP4" s="34"/>
-      <c r="AQ4" s="36"/>
-      <c r="AR4" s="32"/>
-      <c r="AS4" s="34"/>
-      <c r="AT4" s="41"/>
-      <c r="AU4" s="36"/>
-      <c r="AV4" s="32"/>
-      <c r="AW4" s="34"/>
-      <c r="AX4" s="35"/>
-      <c r="AY4" s="36"/>
-      <c r="AZ4" s="32"/>
-      <c r="BA4" s="38"/>
-      <c r="BB4" s="38"/>
-      <c r="BC4" s="38"/>
-      <c r="BD4" s="38"/>
-      <c r="BE4" s="38"/>
-      <c r="BF4" s="38"/>
-      <c r="BG4" s="23"/>
-      <c r="BH4" s="24"/>
-      <c r="BI4" s="25"/>
+      <c r="AL4" s="15"/>
+      <c r="AM4" s="15"/>
+      <c r="AN4" s="15"/>
+      <c r="AO4" s="10"/>
+      <c r="AP4" s="10"/>
+      <c r="AQ4" s="12"/>
+      <c r="AR4" s="35"/>
+      <c r="AS4" s="10"/>
+      <c r="AT4" s="16"/>
+      <c r="AU4" s="12"/>
+      <c r="AV4" s="35"/>
+      <c r="AW4" s="10"/>
+      <c r="AX4" s="11"/>
+      <c r="AY4" s="12"/>
+      <c r="AZ4" s="35"/>
+      <c r="BA4" s="9"/>
+      <c r="BB4" s="9"/>
+      <c r="BC4" s="9"/>
+      <c r="BD4" s="9"/>
+      <c r="BE4" s="9"/>
+      <c r="BF4" s="9"/>
+      <c r="BG4" s="25"/>
+      <c r="BH4" s="26"/>
+      <c r="BI4" s="27"/>
     </row>
     <row r="5" spans="1:61" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
@@ -1561,74 +1666,75 @@
       <c r="G5" t="s">
         <v>53</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" t="e">
+        <f>F5+G5</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I5" t="s">
         <v>55</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>56</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>57</v>
       </c>
-      <c r="K5" t="s">
+      <c r="L5" t="s">
         <v>58</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>59</v>
       </c>
-      <c r="M5" t="s">
+      <c r="N5" t="s">
         <v>60</v>
       </c>
-      <c r="N5" t="s">
+      <c r="O5" t="s">
         <v>61</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" t="s">
         <v>62</v>
       </c>
-      <c r="P5" t="s">
+      <c r="Q5" t="s">
         <v>63</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="R5" t="s">
+        <v>65</v>
+      </c>
+      <c r="S5" t="s">
         <v>64</v>
       </c>
-      <c r="R5" t="s">
+      <c r="T5" t="s">
         <v>66</v>
       </c>
-      <c r="S5" t="s">
-        <v>65</v>
-      </c>
-      <c r="T5" t="s">
+      <c r="U5" t="s">
         <v>67</v>
       </c>
-      <c r="U5" t="s">
+      <c r="V5" t="s">
         <v>68</v>
       </c>
-      <c r="V5" t="s">
+      <c r="W5" t="s">
         <v>69</v>
       </c>
-      <c r="W5" t="s">
+      <c r="X5" t="s">
         <v>70</v>
       </c>
-      <c r="X5" t="s">
+      <c r="Y5" t="s">
         <v>71</v>
       </c>
-      <c r="Y5" t="s">
+      <c r="Z5" t="s">
         <v>72</v>
       </c>
-      <c r="Z5" t="s">
+      <c r="AA5" t="s">
         <v>73</v>
       </c>
-      <c r="AA5" t="s">
+      <c r="AB5" t="s">
         <v>74</v>
       </c>
-      <c r="AB5" t="s">
+      <c r="AC5" t="s">
         <v>75</v>
       </c>
-      <c r="AC5" t="s">
+      <c r="AD5" t="s">
         <v>76</v>
-      </c>
-      <c r="AD5" t="s">
-        <v>77</v>
       </c>
       <c r="AE5" t="s">
         <v>52</v>
@@ -1642,40 +1748,185 @@
         <v>1</v>
       </c>
       <c r="AH5" t="s">
+        <v>77</v>
+      </c>
+      <c r="AI5" t="s">
         <v>78</v>
       </c>
-      <c r="AI5" t="s">
+      <c r="AJ5" t="s">
         <v>79</v>
       </c>
-      <c r="AJ5" t="s">
+      <c r="AK5" t="s">
         <v>80</v>
       </c>
-      <c r="AK5" t="s">
+      <c r="AL5" t="s">
+        <v>80</v>
+      </c>
+      <c r="AM5" t="s">
+        <v>80</v>
+      </c>
+      <c r="AN5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="B6" t="s">
         <v>81</v>
       </c>
-      <c r="AL5" t="s">
-        <v>81</v>
-      </c>
-      <c r="AM5" t="s">
-        <v>81</v>
-      </c>
-      <c r="AN5" t="s">
-        <v>81</v>
+      <c r="C6" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" t="s">
+        <v>83</v>
+      </c>
+      <c r="E6" t="s">
+        <v>84</v>
+      </c>
+      <c r="F6" t="s">
+        <v>85</v>
+      </c>
+      <c r="G6" t="s">
+        <v>86</v>
+      </c>
+      <c r="H6" t="s">
+        <v>87</v>
+      </c>
+      <c r="I6" t="s">
+        <v>88</v>
+      </c>
+      <c r="J6" t="s">
+        <v>89</v>
+      </c>
+      <c r="K6" t="s">
+        <v>90</v>
+      </c>
+      <c r="L6" t="s">
+        <v>91</v>
+      </c>
+      <c r="M6" t="s">
+        <v>92</v>
+      </c>
+      <c r="N6" t="s">
+        <v>93</v>
+      </c>
+      <c r="O6" t="s">
+        <v>94</v>
+      </c>
+      <c r="P6" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>96</v>
+      </c>
+      <c r="R6" t="s">
+        <v>97</v>
+      </c>
+      <c r="S6" t="s">
+        <v>98</v>
+      </c>
+      <c r="T6" t="s">
+        <v>99</v>
+      </c>
+      <c r="U6" t="s">
+        <v>100</v>
+      </c>
+      <c r="V6" t="s">
+        <v>101</v>
+      </c>
+      <c r="W6" t="s">
+        <v>102</v>
+      </c>
+      <c r="X6" t="s">
+        <v>105</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>108</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>103</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>106</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>109</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>104</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="AF9">
+        <v>1</v>
+      </c>
+      <c r="AG9" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:61" x14ac:dyDescent="0.3">
       <c r="H11" s="6"/>
     </row>
+    <row r="12" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="I12" t="s">
+        <v>112</v>
+      </c>
+    </row>
     <row r="13" spans="1:61" x14ac:dyDescent="0.3">
       <c r="G13" s="7"/>
     </row>
+    <row r="14" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="I14" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="18" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I18" t="s">
+        <v>110</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="59">
-    <mergeCell ref="BB3:BB4"/>
-    <mergeCell ref="BC3:BC4"/>
-    <mergeCell ref="BD3:BD4"/>
-    <mergeCell ref="BE3:BE4"/>
-    <mergeCell ref="BF3:BF4"/>
+    <mergeCell ref="AM2:AM4"/>
+    <mergeCell ref="AN2:AN4"/>
+    <mergeCell ref="AO2:AQ2"/>
+    <mergeCell ref="L3:L4"/>
+    <mergeCell ref="M3:M4"/>
+    <mergeCell ref="N3:N4"/>
+    <mergeCell ref="O3:O4"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="D2:D4"/>
+    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="AI3:AI4"/>
+    <mergeCell ref="AJ3:AJ4"/>
+    <mergeCell ref="AK3:AK4"/>
+    <mergeCell ref="P3:P4"/>
+    <mergeCell ref="Q3:S3"/>
+    <mergeCell ref="T3:V3"/>
+    <mergeCell ref="W3:Y3"/>
+    <mergeCell ref="Z3:AB3"/>
+    <mergeCell ref="AC3:AE3"/>
+    <mergeCell ref="BD2:BF2"/>
+    <mergeCell ref="BG2:BG4"/>
+    <mergeCell ref="BH2:BH4"/>
+    <mergeCell ref="BI2:BI4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="AR2:AR4"/>
+    <mergeCell ref="AS2:AU2"/>
+    <mergeCell ref="AV2:AV4"/>
+    <mergeCell ref="AW2:AY2"/>
+    <mergeCell ref="AZ2:AZ4"/>
+    <mergeCell ref="BA2:BC2"/>
     <mergeCell ref="AW3:AW4"/>
     <mergeCell ref="AX3:AX4"/>
     <mergeCell ref="AY3:AY4"/>
@@ -1692,44 +1943,11 @@
     <mergeCell ref="AF3:AF4"/>
     <mergeCell ref="AG3:AG4"/>
     <mergeCell ref="AH3:AH4"/>
-    <mergeCell ref="BD2:BF2"/>
-    <mergeCell ref="BG2:BG4"/>
-    <mergeCell ref="BH2:BH4"/>
-    <mergeCell ref="BI2:BI4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="I3:I4"/>
-    <mergeCell ref="J3:J4"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="AR2:AR4"/>
-    <mergeCell ref="AS2:AU2"/>
-    <mergeCell ref="AV2:AV4"/>
-    <mergeCell ref="AW2:AY2"/>
-    <mergeCell ref="AZ2:AZ4"/>
-    <mergeCell ref="BA2:BC2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="AI3:AI4"/>
-    <mergeCell ref="AJ3:AJ4"/>
-    <mergeCell ref="AK3:AK4"/>
-    <mergeCell ref="P3:P4"/>
-    <mergeCell ref="Q3:S3"/>
-    <mergeCell ref="T3:V3"/>
-    <mergeCell ref="W3:Y3"/>
-    <mergeCell ref="Z3:AB3"/>
-    <mergeCell ref="AC3:AE3"/>
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="B2:B4"/>
-    <mergeCell ref="C2:C4"/>
-    <mergeCell ref="D2:D4"/>
-    <mergeCell ref="E2:E4"/>
-    <mergeCell ref="AM2:AM4"/>
-    <mergeCell ref="AN2:AN4"/>
-    <mergeCell ref="AO2:AQ2"/>
-    <mergeCell ref="L3:L4"/>
-    <mergeCell ref="M3:M4"/>
-    <mergeCell ref="N3:N4"/>
-    <mergeCell ref="O3:O4"/>
+    <mergeCell ref="BB3:BB4"/>
+    <mergeCell ref="BC3:BC4"/>
+    <mergeCell ref="BD3:BD4"/>
+    <mergeCell ref="BE3:BE4"/>
+    <mergeCell ref="BF3:BF4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967292" r:id="rId1"/>

</xml_diff>

<commit_message>
add more help labels on xls
</commit_message>
<xml_diff>
--- a/api/templates/results_10a_10b_covid_ntp_use/en.xlsx
+++ b/api/templates/results_10a_10b_covid_ntp_use/en.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu-20.04\home\maiki\.oh-my-zsh\aspect\api\templates\results_10a_10b_covid_ntp_use\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5AFEC5A-AF90-4F0F-B58C-58570DDA85B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93BD1658-BCC1-4C27-B82C-3C313FE4B8A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="6264" windowWidth="8856" windowHeight="4632" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="January" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="136">
   <si>
     <t>Sl No.</t>
   </si>
@@ -296,9 +296,6 @@
     <t>&lt;smearPrev&gt;</t>
   </si>
   <si>
-    <t>&lt;sumMe&gt;</t>
-  </si>
-  <si>
     <t>c6</t>
   </si>
   <si>
@@ -311,15 +308,9 @@
     <t>nombres aca</t>
   </si>
   <si>
-    <t>b26-26-32</t>
-  </si>
-  <si>
     <t>c26-29-32</t>
   </si>
   <si>
-    <t>f5+g5</t>
-  </si>
-  <si>
     <t>e26-29-32</t>
   </si>
   <si>
@@ -344,9 +335,6 @@
     <t>l26-29-32</t>
   </si>
   <si>
-    <t>026-29-32</t>
-  </si>
-  <si>
     <t>o27-30-33</t>
   </si>
   <si>
@@ -389,10 +377,91 @@
     <t>E26+F26+G26+H26+I26+J26+K26+L26+O26+O27+O28+R26+R27+R28+S26</t>
   </si>
   <si>
-    <t>O26+O27+O28+R26+R27+R28+S26</t>
-  </si>
-  <si>
     <t>i5+j5+k5+l5+m5+n5+o5+p5+q5+r5+s5+t5+u5+v5</t>
+  </si>
+  <si>
+    <t>S26</t>
+  </si>
+  <si>
+    <t>B39+C39+D39</t>
+  </si>
+  <si>
+    <t>b39-31-43</t>
+  </si>
+  <si>
+    <t>d39-41-43</t>
+  </si>
+  <si>
+    <t>c39-41-43</t>
+  </si>
+  <si>
+    <t>o26-29-32</t>
+  </si>
+  <si>
+    <t>b26-29-32</t>
+  </si>
+  <si>
+    <t>h5+ak5</t>
+  </si>
+  <si>
+    <t>u26</t>
+  </si>
+  <si>
+    <t>h12</t>
+  </si>
+  <si>
+    <t>h13</t>
+  </si>
+  <si>
+    <t>h14</t>
+  </si>
+  <si>
+    <t>D29+E41-D32-E43</t>
+  </si>
+  <si>
+    <t>D17</t>
+  </si>
+  <si>
+    <t>d26</t>
+  </si>
+  <si>
+    <t>b26+c26</t>
+  </si>
+  <si>
+    <t>.</t>
+  </si>
+  <si>
+    <t>Necesito fila 2!</t>
+  </si>
+  <si>
+    <t>Necesito fila 3!</t>
+  </si>
+  <si>
+    <t>D20</t>
+  </si>
+  <si>
+    <t>H12-D29-E41</t>
+  </si>
+  <si>
+    <t>?? No hay datos rpt ruslan</t>
+  </si>
+  <si>
+    <t>D18</t>
+  </si>
+  <si>
+    <t>D32+E43</t>
+  </si>
+  <si>
+    <t>D19</t>
+  </si>
+  <si>
+    <t>??</t>
+  </si>
+  <si>
+    <t>E17</t>
+  </si>
+  <si>
+    <t>U29-U32</t>
   </si>
 </sst>
 </file>
@@ -1273,6 +1342,7 @@
     <col min="2" max="2" width="13.6640625" customWidth="1"/>
     <col min="3" max="3" width="16.5546875" customWidth="1"/>
     <col min="4" max="4" width="31.33203125" customWidth="1"/>
+    <col min="5" max="5" width="11.77734375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="21.109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.88671875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.21875" bestFit="1" customWidth="1"/>
@@ -1284,7 +1354,8 @@
     <col min="21" max="21" width="10.6640625" customWidth="1"/>
     <col min="22" max="22" width="10.77734375" customWidth="1"/>
     <col min="23" max="23" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="13.33203125" customWidth="1"/>
+    <col min="25" max="25" width="13.44140625" customWidth="1"/>
     <col min="26" max="26" width="19.88671875" bestFit="1" customWidth="1"/>
     <col min="27" max="28" width="15.44140625" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="19.109375" bestFit="1" customWidth="1"/>
@@ -1292,8 +1363,10 @@
     <col min="31" max="31" width="8.44140625" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="10.109375" customWidth="1"/>
     <col min="33" max="33" width="9.109375" customWidth="1"/>
-    <col min="34" max="34" width="10.109375" customWidth="1"/>
-    <col min="35" max="45" width="9.109375" customWidth="1"/>
+    <col min="34" max="34" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="13.77734375" customWidth="1"/>
+    <col min="38" max="45" width="9.109375" customWidth="1"/>
     <col min="46" max="46" width="9.109375" style="4" customWidth="1"/>
     <col min="47" max="48" width="9.109375" customWidth="1"/>
     <col min="50" max="50" width="9.109375" style="5"/>
@@ -1743,9 +1816,9 @@
         <f>W5+X5+Y5</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AG5">
-        <f>IF(MOD(ROW()-5,3) =0, 1,0)</f>
-        <v>1</v>
+      <c r="AG5" t="e">
+        <f>IF(MOD(ROW()-5,3) =0, SUM(I5+J5+K5+L5+M5+N5+O5+P5+Q5+R5+S5+T5+U5+V5),0)</f>
+        <v>#VALUE!</v>
       </c>
       <c r="AH5" t="s">
         <v>77</v>
@@ -1756,114 +1829,190 @@
       <c r="AJ5" t="s">
         <v>79</v>
       </c>
-      <c r="AK5" t="s">
-        <v>80</v>
-      </c>
-      <c r="AL5" t="s">
-        <v>80</v>
-      </c>
-      <c r="AM5" t="s">
-        <v>80</v>
-      </c>
-      <c r="AN5" t="s">
-        <v>80</v>
+      <c r="AK5">
+        <f>IF(MOD(ROW()-5,3) =0, SUM(AH5,AI5,AJ5),0)</f>
+        <v>0</v>
+      </c>
+      <c r="AL5" t="e">
+        <f>IF(MOD(ROW()-5,3) =0, SUM(H5+AK5),0)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="AM5" t="e">
+        <f>AG5</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="AN5" t="e">
+        <f>+AL5+AM5</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="AO5" t="s">
+        <v>125</v>
+      </c>
+      <c r="AP5" t="s">
+        <v>126</v>
+      </c>
+      <c r="AQ5" t="s">
+        <v>129</v>
+      </c>
+      <c r="AR5" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="6" spans="1:61" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" t="s">
         <v>81</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>82</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>83</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
+        <v>114</v>
+      </c>
+      <c r="G6" t="s">
         <v>84</v>
       </c>
-      <c r="F6" t="s">
+      <c r="H6" t="s">
+        <v>122</v>
+      </c>
+      <c r="I6" t="s">
         <v>85</v>
       </c>
-      <c r="G6" t="s">
+      <c r="J6" t="s">
         <v>86</v>
       </c>
-      <c r="H6" t="s">
+      <c r="K6" t="s">
         <v>87</v>
       </c>
-      <c r="I6" t="s">
+      <c r="L6" t="s">
         <v>88</v>
       </c>
-      <c r="J6" t="s">
+      <c r="M6" t="s">
         <v>89</v>
       </c>
-      <c r="K6" t="s">
+      <c r="N6" t="s">
         <v>90</v>
       </c>
-      <c r="L6" t="s">
+      <c r="O6" t="s">
         <v>91</v>
       </c>
-      <c r="M6" t="s">
+      <c r="P6" t="s">
         <v>92</v>
       </c>
-      <c r="N6" t="s">
+      <c r="Q6" t="s">
+        <v>113</v>
+      </c>
+      <c r="R6" t="s">
         <v>93</v>
       </c>
-      <c r="O6" t="s">
+      <c r="S6" t="s">
         <v>94</v>
       </c>
-      <c r="P6" t="s">
+      <c r="T6" t="s">
         <v>95</v>
       </c>
-      <c r="Q6" t="s">
+      <c r="U6" t="s">
         <v>96</v>
       </c>
-      <c r="R6" t="s">
+      <c r="V6" t="s">
         <v>97</v>
       </c>
-      <c r="S6" t="s">
+      <c r="W6" t="s">
         <v>98</v>
       </c>
-      <c r="T6" t="s">
+      <c r="X6" t="s">
+        <v>101</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>104</v>
+      </c>
+      <c r="Z6" t="s">
         <v>99</v>
       </c>
-      <c r="U6" t="s">
+      <c r="AA6" t="s">
+        <v>102</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>105</v>
+      </c>
+      <c r="AC6" t="s">
         <v>100</v>
       </c>
-      <c r="V6" t="s">
-        <v>101</v>
-      </c>
-      <c r="W6" t="s">
-        <v>102</v>
-      </c>
-      <c r="X6" t="s">
-        <v>105</v>
-      </c>
-      <c r="Y6" t="s">
-        <v>108</v>
-      </c>
-      <c r="Z6" t="s">
+      <c r="AD6" t="s">
         <v>103</v>
       </c>
-      <c r="AA6" t="s">
+      <c r="AG6" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH6" t="s">
+        <v>110</v>
+      </c>
+      <c r="AI6" t="s">
+        <v>112</v>
+      </c>
+      <c r="AJ6" t="s">
+        <v>111</v>
+      </c>
+      <c r="AK6" t="s">
+        <v>109</v>
+      </c>
+      <c r="AL6" t="s">
+        <v>117</v>
+      </c>
+      <c r="AM6" t="s">
+        <v>118</v>
+      </c>
+      <c r="AN6" t="s">
+        <v>119</v>
+      </c>
+      <c r="AO6" t="s">
+        <v>121</v>
+      </c>
+      <c r="AP6" t="s">
+        <v>130</v>
+      </c>
+      <c r="AQ6" t="s">
+        <v>132</v>
+      </c>
+      <c r="AR6" t="s">
+        <v>127</v>
+      </c>
+      <c r="AS6" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="7" spans="1:61" x14ac:dyDescent="0.3">
+      <c r="H7" t="s">
+        <v>123</v>
+      </c>
+      <c r="AG7" t="s">
         <v>106</v>
       </c>
-      <c r="AB6" t="s">
-        <v>109</v>
-      </c>
-      <c r="AC6" t="s">
-        <v>104</v>
-      </c>
-      <c r="AD6" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="9" spans="1:61" x14ac:dyDescent="0.3">
-      <c r="AF9">
-        <v>1</v>
-      </c>
-      <c r="AG9" t="s">
-        <v>110</v>
+      <c r="AH7" t="s">
+        <v>124</v>
+      </c>
+      <c r="AL7" t="s">
+        <v>115</v>
+      </c>
+      <c r="AO7" t="s">
+        <v>120</v>
+      </c>
+      <c r="AP7" t="s">
+        <v>131</v>
+      </c>
+      <c r="AQ7" t="s">
+        <v>133</v>
+      </c>
+      <c r="AR7" t="s">
+        <v>128</v>
+      </c>
+      <c r="AS7" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="11" spans="1:61" x14ac:dyDescent="0.3">
@@ -1871,7 +2020,7 @@
     </row>
     <row r="12" spans="1:61" x14ac:dyDescent="0.3">
       <c r="I12" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="13" spans="1:61" x14ac:dyDescent="0.3">
@@ -1879,12 +2028,12 @@
     </row>
     <row r="14" spans="1:61" x14ac:dyDescent="0.3">
       <c r="I14" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="18" spans="9:9" x14ac:dyDescent="0.3">
       <c r="I18" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add missing tags on xls and mapping
</commit_message>
<xml_diff>
--- a/api/templates/results_10a_10b_covid_ntp_use/en.xlsx
+++ b/api/templates/results_10a_10b_covid_ntp_use/en.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu-20.04\home\maiki\.oh-my-zsh\aspect\api\templates\results_10a_10b_covid_ntp_use\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ACAD918-B1C0-45C9-9926-A2E2BCC0C5E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA27C885-52F3-4B59-87AF-5A35FFB17E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="6708" windowWidth="7080" windowHeight="3708" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="January" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="88">
   <si>
     <t>Sl No.</t>
   </si>
@@ -296,220 +296,28 @@
     <t>&lt;smearPrev&gt;</t>
   </si>
   <si>
-    <t>c6</t>
-  </si>
-  <si>
-    <t>c7</t>
-  </si>
-  <si>
-    <t>c8</t>
-  </si>
-  <si>
-    <t>nombres aca</t>
-  </si>
-  <si>
-    <t>c26-29-32</t>
-  </si>
-  <si>
-    <t>e26-29-32</t>
-  </si>
-  <si>
-    <t>f26-29-32</t>
-  </si>
-  <si>
-    <t>g26-29-32</t>
-  </si>
-  <si>
-    <t>h26-29-32</t>
-  </si>
-  <si>
-    <t>i26-29-32</t>
-  </si>
-  <si>
-    <t>j26-29-32</t>
-  </si>
-  <si>
-    <t>k26-29-32</t>
-  </si>
-  <si>
-    <t>l26-29-32</t>
-  </si>
-  <si>
-    <t>o27-30-33</t>
-  </si>
-  <si>
-    <t>o28-31-34</t>
-  </si>
-  <si>
-    <t>r26-29-32</t>
-  </si>
-  <si>
-    <t>R27-30-33</t>
-  </si>
-  <si>
-    <t>r28-31-34</t>
-  </si>
-  <si>
-    <t>m40-p40-s40</t>
-  </si>
-  <si>
-    <t>m41-p41-s41</t>
-  </si>
-  <si>
-    <t>m42-p42-s42</t>
-  </si>
-  <si>
-    <t>n40-q40-t40</t>
-  </si>
-  <si>
-    <t>n41-q41-t41</t>
-  </si>
-  <si>
-    <t>n42-q42-t42</t>
-  </si>
-  <si>
-    <t>o41-r40-u40</t>
-  </si>
-  <si>
-    <t>o41-r41-u41</t>
-  </si>
-  <si>
-    <t>E26+F26+G26+H26+I26+J26+K26+L26+O26+O27+O28+R26+R27+R28+S26</t>
-  </si>
-  <si>
-    <t>B39+C39+D39</t>
-  </si>
-  <si>
-    <t>b39-31-43</t>
-  </si>
-  <si>
-    <t>d39-41-43</t>
-  </si>
-  <si>
-    <t>c39-41-43</t>
-  </si>
-  <si>
-    <t>o26-29-32</t>
-  </si>
-  <si>
-    <t>b26-29-32</t>
-  </si>
-  <si>
-    <t>h5+ak5</t>
-  </si>
-  <si>
-    <t>u26</t>
-  </si>
-  <si>
-    <t>h12</t>
-  </si>
-  <si>
-    <t>h13</t>
-  </si>
-  <si>
-    <t>h14</t>
-  </si>
-  <si>
-    <t>D29+E41-D32-E43</t>
-  </si>
-  <si>
-    <t>D17</t>
-  </si>
-  <si>
-    <t>d26</t>
-  </si>
-  <si>
-    <t>b26+c26</t>
-  </si>
-  <si>
-    <t>.</t>
-  </si>
-  <si>
-    <t>Necesito fila 2!</t>
-  </si>
-  <si>
-    <t>Necesito fila 3!</t>
-  </si>
-  <si>
-    <t>D20</t>
-  </si>
-  <si>
-    <t>H12-D29-E41</t>
-  </si>
-  <si>
-    <t>?? No hay datos rpt ruslan</t>
-  </si>
-  <si>
-    <t>D18</t>
-  </si>
-  <si>
-    <t>D32+E43</t>
-  </si>
-  <si>
-    <t>D19</t>
-  </si>
-  <si>
-    <t>??</t>
-  </si>
-  <si>
-    <t>E17</t>
-  </si>
-  <si>
-    <t>U29-U32</t>
-  </si>
-  <si>
-    <t>Necesito fila 2</t>
-  </si>
-  <si>
-    <t>E18</t>
-  </si>
-  <si>
-    <t>U32</t>
-  </si>
-  <si>
-    <t>E19</t>
-  </si>
-  <si>
-    <t>E20</t>
-  </si>
-  <si>
-    <t>F17</t>
-  </si>
-  <si>
-    <t>F18</t>
-  </si>
-  <si>
-    <t>F19</t>
-  </si>
-  <si>
-    <t>F20</t>
-  </si>
-  <si>
-    <t>L18</t>
-  </si>
-  <si>
-    <t>M18</t>
-  </si>
-  <si>
-    <t>N18</t>
-  </si>
-  <si>
-    <t>O18</t>
-  </si>
-  <si>
-    <t>P18</t>
-  </si>
-  <si>
-    <t>Q18</t>
-  </si>
-  <si>
-    <t>R18</t>
-  </si>
-  <si>
-    <t>H13-U29</t>
-  </si>
-  <si>
-    <t>AG5</t>
+    <t>&lt;presumtiveTbIndeterminated&gt;</t>
+  </si>
+  <si>
+    <t>&lt;presumtiveDrTbIndeterminated&gt;</t>
+  </si>
+  <si>
+    <t>&lt;presumptiveTbInvalid&gt;</t>
+  </si>
+  <si>
+    <t>&lt;presumptiveTbNoResult&gt;</t>
+  </si>
+  <si>
+    <t>&lt;presumptiveDrTbInvalid&gt;</t>
+  </si>
+  <si>
+    <t>&lt;presumptiveDrTbNoResult&gt;</t>
+  </si>
+  <si>
+    <t>&lt;presumptiveDrTbError&gt;</t>
+  </si>
+  <si>
+    <t>&lt;deviceName&gt;</t>
   </si>
 </sst>
 </file>
@@ -520,7 +328,7 @@
     <numFmt numFmtId="164" formatCode="[$-409]General"/>
     <numFmt numFmtId="165" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -647,14 +455,6 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -869,7 +669,7 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="17" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection hidden="1"/>
@@ -884,7 +684,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
@@ -1382,7 +1184,7 @@
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="A1:BI13"/>
+  <dimension ref="A1:BI5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.6640625" customWidth="1"/>
@@ -1417,6 +1219,8 @@
     <col min="46" max="46" width="9.109375" style="4" customWidth="1"/>
     <col min="47" max="48" width="9.109375" customWidth="1"/>
     <col min="50" max="50" width="9.109375" style="5"/>
+    <col min="51" max="52" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="21.88671875" bestFit="1" customWidth="1"/>
     <col min="60" max="60" width="13.5546875" customWidth="1"/>
     <col min="61" max="61" width="9.109375" customWidth="1"/>
   </cols>
@@ -1430,264 +1234,264 @@
       </c>
     </row>
     <row r="2" spans="1:61" s="1" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="39" t="s">
+      <c r="C2" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="40"/>
-      <c r="F2" s="36" t="s">
+      <c r="E2" s="42"/>
+      <c r="F2" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="12" t="s">
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
+      <c r="I2" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="12"/>
-      <c r="P2" s="12"/>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="12"/>
-      <c r="S2" s="12"/>
-      <c r="T2" s="12"/>
-      <c r="U2" s="12"/>
-      <c r="V2" s="12"/>
-      <c r="W2" s="12"/>
-      <c r="X2" s="12"/>
-      <c r="Y2" s="12"/>
-      <c r="Z2" s="12"/>
-      <c r="AA2" s="12"/>
-      <c r="AB2" s="12"/>
-      <c r="AC2" s="12"/>
-      <c r="AD2" s="12"/>
-      <c r="AE2" s="12"/>
-      <c r="AF2" s="12"/>
-      <c r="AG2" s="12"/>
-      <c r="AH2" s="13" t="s">
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="14"/>
+      <c r="P2" s="14"/>
+      <c r="Q2" s="14"/>
+      <c r="R2" s="14"/>
+      <c r="S2" s="14"/>
+      <c r="T2" s="14"/>
+      <c r="U2" s="14"/>
+      <c r="V2" s="14"/>
+      <c r="W2" s="14"/>
+      <c r="X2" s="14"/>
+      <c r="Y2" s="14"/>
+      <c r="Z2" s="14"/>
+      <c r="AA2" s="14"/>
+      <c r="AB2" s="14"/>
+      <c r="AC2" s="14"/>
+      <c r="AD2" s="14"/>
+      <c r="AE2" s="14"/>
+      <c r="AF2" s="14"/>
+      <c r="AG2" s="14"/>
+      <c r="AH2" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="AI2" s="13"/>
-      <c r="AJ2" s="13"/>
-      <c r="AK2" s="13"/>
-      <c r="AL2" s="14" t="s">
+      <c r="AI2" s="15"/>
+      <c r="AJ2" s="15"/>
+      <c r="AK2" s="15"/>
+      <c r="AL2" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="AM2" s="14" t="s">
+      <c r="AM2" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="AN2" s="14" t="s">
+      <c r="AN2" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="AO2" s="20" t="s">
+      <c r="AO2" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="AP2" s="21"/>
-      <c r="AQ2" s="21"/>
-      <c r="AR2" s="32" t="s">
+      <c r="AP2" s="23"/>
+      <c r="AQ2" s="23"/>
+      <c r="AR2" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="AS2" s="20" t="s">
+      <c r="AS2" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="AT2" s="21"/>
-      <c r="AU2" s="21"/>
-      <c r="AV2" s="32" t="s">
+      <c r="AT2" s="23"/>
+      <c r="AU2" s="23"/>
+      <c r="AV2" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="AW2" s="20" t="s">
+      <c r="AW2" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="AX2" s="21"/>
-      <c r="AY2" s="21"/>
-      <c r="AZ2" s="32" t="s">
+      <c r="AX2" s="23"/>
+      <c r="AY2" s="23"/>
+      <c r="AZ2" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="BA2" s="20" t="s">
+      <c r="BA2" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="BB2" s="21"/>
-      <c r="BC2" s="35"/>
-      <c r="BD2" s="20" t="s">
+      <c r="BB2" s="23"/>
+      <c r="BC2" s="37"/>
+      <c r="BD2" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="BE2" s="21"/>
-      <c r="BF2" s="21"/>
-      <c r="BG2" s="22" t="s">
+      <c r="BE2" s="23"/>
+      <c r="BF2" s="23"/>
+      <c r="BG2" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="BH2" s="25" t="s">
+      <c r="BH2" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="BI2" s="26" t="s">
+      <c r="BI2" s="28" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:61" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="38"/>
-      <c r="B3" s="39"/>
-      <c r="C3" s="39"/>
-      <c r="D3" s="39"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="27" t="s">
+      <c r="A3" s="40"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="29" t="s">
+      <c r="G3" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="30" t="s">
+      <c r="H3" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="31" t="s">
+      <c r="I3" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="J3" s="31" t="s">
+      <c r="J3" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="K3" s="31" t="s">
+      <c r="K3" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="L3" s="31" t="s">
+      <c r="L3" s="33" t="s">
         <v>27</v>
       </c>
-      <c r="M3" s="31" t="s">
+      <c r="M3" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="N3" s="31" t="s">
+      <c r="N3" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="O3" s="31" t="s">
+      <c r="O3" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="P3" s="31" t="s">
+      <c r="P3" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="Q3" s="31" t="s">
+      <c r="Q3" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="R3" s="31"/>
-      <c r="S3" s="31"/>
-      <c r="T3" s="31" t="s">
+      <c r="R3" s="33"/>
+      <c r="S3" s="33"/>
+      <c r="T3" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="U3" s="31"/>
-      <c r="V3" s="31"/>
-      <c r="W3" s="37" t="s">
+      <c r="U3" s="33"/>
+      <c r="V3" s="33"/>
+      <c r="W3" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="X3" s="37"/>
-      <c r="Y3" s="37"/>
-      <c r="Z3" s="37" t="s">
+      <c r="X3" s="39"/>
+      <c r="Y3" s="39"/>
+      <c r="Z3" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="AA3" s="37"/>
-      <c r="AB3" s="37"/>
-      <c r="AC3" s="37" t="s">
+      <c r="AA3" s="39"/>
+      <c r="AB3" s="39"/>
+      <c r="AC3" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="AD3" s="37"/>
-      <c r="AE3" s="37"/>
-      <c r="AF3" s="16" t="s">
+      <c r="AD3" s="39"/>
+      <c r="AE3" s="39"/>
+      <c r="AF3" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="AG3" s="18" t="s">
+      <c r="AG3" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="AH3" s="19" t="s">
+      <c r="AH3" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="AI3" s="19" t="s">
+      <c r="AI3" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="AJ3" s="19" t="s">
+      <c r="AJ3" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="AK3" s="18" t="s">
+      <c r="AK3" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="AL3" s="14"/>
-      <c r="AM3" s="14"/>
-      <c r="AN3" s="14"/>
-      <c r="AO3" s="9" t="s">
+      <c r="AL3" s="16"/>
+      <c r="AM3" s="16"/>
+      <c r="AN3" s="16"/>
+      <c r="AO3" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="AP3" s="9" t="s">
+      <c r="AP3" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="AQ3" s="11" t="s">
+      <c r="AQ3" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="AR3" s="33"/>
-      <c r="AS3" s="9" t="s">
+      <c r="AR3" s="35"/>
+      <c r="AS3" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="AT3" s="15" t="s">
+      <c r="AT3" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="AU3" s="11" t="s">
+      <c r="AU3" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="AV3" s="33"/>
-      <c r="AW3" s="9" t="s">
+      <c r="AV3" s="35"/>
+      <c r="AW3" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="AX3" s="10" t="s">
+      <c r="AX3" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="AY3" s="11" t="s">
+      <c r="AY3" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="AZ3" s="33"/>
-      <c r="BA3" s="7" t="s">
+      <c r="AZ3" s="35"/>
+      <c r="BA3" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="BB3" s="7" t="s">
+      <c r="BB3" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="BC3" s="7" t="s">
+      <c r="BC3" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="BD3" s="7" t="s">
+      <c r="BD3" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="BE3" s="7" t="s">
+      <c r="BE3" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="BF3" s="7" t="s">
+      <c r="BF3" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="BG3" s="23"/>
-      <c r="BH3" s="25"/>
-      <c r="BI3" s="26"/>
+      <c r="BG3" s="25"/>
+      <c r="BH3" s="27"/>
+      <c r="BI3" s="28"/>
     </row>
     <row r="4" spans="1:61" s="1" customFormat="1" ht="44.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="38"/>
-      <c r="B4" s="39"/>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="29"/>
-      <c r="H4" s="30"/>
-      <c r="I4" s="31"/>
-      <c r="J4" s="31"/>
-      <c r="K4" s="31"/>
-      <c r="L4" s="31"/>
-      <c r="M4" s="31"/>
-      <c r="N4" s="31"/>
-      <c r="O4" s="31"/>
-      <c r="P4" s="31"/>
+      <c r="A4" s="40"/>
+      <c r="B4" s="41"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="44"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="33"/>
+      <c r="J4" s="33"/>
+      <c r="K4" s="33"/>
+      <c r="L4" s="33"/>
+      <c r="M4" s="33"/>
+      <c r="N4" s="33"/>
+      <c r="O4" s="33"/>
+      <c r="P4" s="33"/>
       <c r="Q4" s="2" t="s">
         <v>45</v>
       </c>
@@ -1733,38 +1537,38 @@
       <c r="AE4" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AF4" s="17"/>
-      <c r="AG4" s="18"/>
-      <c r="AH4" s="19"/>
-      <c r="AI4" s="19"/>
-      <c r="AJ4" s="19"/>
-      <c r="AK4" s="18"/>
-      <c r="AL4" s="14"/>
-      <c r="AM4" s="14"/>
-      <c r="AN4" s="14"/>
-      <c r="AO4" s="9"/>
-      <c r="AP4" s="9"/>
-      <c r="AQ4" s="11"/>
-      <c r="AR4" s="34"/>
-      <c r="AS4" s="9"/>
-      <c r="AT4" s="15"/>
-      <c r="AU4" s="11"/>
-      <c r="AV4" s="34"/>
-      <c r="AW4" s="9"/>
-      <c r="AX4" s="10"/>
-      <c r="AY4" s="11"/>
-      <c r="AZ4" s="34"/>
-      <c r="BA4" s="8"/>
-      <c r="BB4" s="8"/>
-      <c r="BC4" s="8"/>
-      <c r="BD4" s="8"/>
-      <c r="BE4" s="8"/>
-      <c r="BF4" s="8"/>
-      <c r="BG4" s="24"/>
-      <c r="BH4" s="25"/>
-      <c r="BI4" s="26"/>
+      <c r="AF4" s="19"/>
+      <c r="AG4" s="20"/>
+      <c r="AH4" s="21"/>
+      <c r="AI4" s="21"/>
+      <c r="AJ4" s="21"/>
+      <c r="AK4" s="20"/>
+      <c r="AL4" s="16"/>
+      <c r="AM4" s="16"/>
+      <c r="AN4" s="16"/>
+      <c r="AO4" s="11"/>
+      <c r="AP4" s="11"/>
+      <c r="AQ4" s="13"/>
+      <c r="AR4" s="36"/>
+      <c r="AS4" s="11"/>
+      <c r="AT4" s="17"/>
+      <c r="AU4" s="13"/>
+      <c r="AV4" s="36"/>
+      <c r="AW4" s="11"/>
+      <c r="AX4" s="12"/>
+      <c r="AY4" s="13"/>
+      <c r="AZ4" s="36"/>
+      <c r="BA4" s="10"/>
+      <c r="BB4" s="10"/>
+      <c r="BC4" s="10"/>
+      <c r="BD4" s="10"/>
+      <c r="BE4" s="10"/>
+      <c r="BF4" s="10"/>
+      <c r="BG4" s="26"/>
+      <c r="BH4" s="27"/>
+      <c r="BI4" s="28"/>
     </row>
-    <row r="5" spans="1:61" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:61" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>48</v>
       </c>
@@ -1778,7 +1582,7 @@
         <v>49</v>
       </c>
       <c r="E5" t="s">
-        <v>52</v>
+        <v>87</v>
       </c>
       <c r="F5" t="s">
         <v>54</v>
@@ -1786,7 +1590,7 @@
       <c r="G5" t="s">
         <v>53</v>
       </c>
-      <c r="H5" t="e">
+      <c r="H5" s="6" t="e">
         <f>F5+G5</f>
         <v>#VALUE!</v>
       </c>
@@ -1859,13 +1663,13 @@
       <c r="AE5" t="s">
         <v>52</v>
       </c>
-      <c r="AF5" t="e">
-        <f>W5+X5+Y5</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="AG5" t="e">
-        <f>IF(MOD(ROW()-5,3) =0, SUM(I5+J5+K5+L5+M5+N5+O5+P5+Q5+R5+S5+T5+U5+V5),0)</f>
-        <v>#VALUE!</v>
+      <c r="AF5" s="6">
+        <f>SUM(W5:AD5)</f>
+        <v>0</v>
+      </c>
+      <c r="AG5" s="6">
+        <f>SUM(I5:V5)</f>
+        <v>0</v>
       </c>
       <c r="AH5" t="s">
         <v>77</v>
@@ -1876,267 +1680,87 @@
       <c r="AJ5" t="s">
         <v>79</v>
       </c>
-      <c r="AK5">
-        <f>IF(MOD(ROW()-5,3) =0, SUM(AH5,AI5,AJ5),0)</f>
+      <c r="AK5" s="6">
+        <f>SUM(AH5:AJ5)</f>
         <v>0</v>
       </c>
-      <c r="AL5" t="e">
-        <f>IF(MOD(ROW()-5,3) =0, SUM(H5+AK5),0)</f>
+      <c r="AL5" s="6" t="e">
+        <f>IF(MOD(ROW()-5,3) =0, SUM(H5+AK5),"")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AM5" t="e">
-        <f>AG5</f>
+      <c r="AM5" s="6">
+        <f>IF(MOD(ROW()-5,3) =0, AG5,"")</f>
+        <v>0</v>
+      </c>
+      <c r="AN5" s="6" t="e">
+        <f>IF(MOD(ROW()-5,3) =0, AL5+AM5,"")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AN5" t="e">
-        <f>+AL5+AM5</f>
+      <c r="AO5" s="6">
+        <f>IF(MOD(ROW()-5,3) =0, H6+AK6-H7-AK7,"")</f>
+        <v>0</v>
+      </c>
+      <c r="AP5" s="6">
+        <f>IF(MOD(ROW()-5,3) =0, H7+AK7,"")</f>
+        <v>0</v>
+      </c>
+      <c r="AQ5" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="AR5" s="6" t="e">
+        <f>IF(MOD(ROW()-5,3) =0,AL5-H6-AK6,"")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AO5" t="s">
-        <v>123</v>
-      </c>
-      <c r="AP5" t="s">
-        <v>124</v>
-      </c>
-      <c r="AQ5" t="s">
-        <v>127</v>
-      </c>
-      <c r="AR5" t="s">
-        <v>123</v>
-      </c>
-      <c r="AS5" t="s">
-        <v>134</v>
-      </c>
-      <c r="AT5" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="AU5" t="s">
-        <v>127</v>
-      </c>
-      <c r="AV5" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="6" spans="1:61" x14ac:dyDescent="0.3">
-      <c r="B6" t="s">
-        <v>80</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="AS5" s="6">
+        <f>IF(MOD(ROW()-5,3) =0,AG6-AG7,"")</f>
+        <v>0</v>
+      </c>
+      <c r="AT5" s="7">
+        <f>IF(MOD(ROW()-5,3) =0,AG7,"")</f>
+        <v>0</v>
+      </c>
+      <c r="AU5" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="D6" t="s">
+      <c r="AV5" s="6">
+        <f>AG5-AG6</f>
+        <v>0</v>
+      </c>
+      <c r="AW5" s="6">
+        <f>IF(MOD(ROW()-5,3)=0,AO5+AS5,"")</f>
+        <v>0</v>
+      </c>
+      <c r="AX5" s="8">
+        <f>IF(MOD(ROW()-5,3)=0,AP5+AT5,"")</f>
+        <v>0</v>
+      </c>
+      <c r="AY5" s="6" t="e">
+        <f>IF(MOD(ROW()-5,3)=0,AQ5+AU5,"")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="AZ5" s="6" t="e">
+        <f>IF(MOD(ROW()-5,3) =0,AR5+AV5,"")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="BA5" t="s">
         <v>82</v>
       </c>
-      <c r="E6" t="s">
+      <c r="BB5" t="s">
         <v>83</v>
       </c>
-      <c r="F6" t="s">
-        <v>112</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="BD5" t="s">
         <v>84</v>
       </c>
-      <c r="H6">
-        <v>6000</v>
-      </c>
-      <c r="I6" t="s">
+      <c r="BE5" t="s">
         <v>85</v>
       </c>
-      <c r="J6" t="s">
+      <c r="BF5" t="s">
         <v>86</v>
       </c>
-      <c r="K6" t="s">
-        <v>87</v>
-      </c>
-      <c r="L6" t="s">
-        <v>88</v>
-      </c>
-      <c r="M6" t="s">
-        <v>89</v>
-      </c>
-      <c r="N6" t="s">
-        <v>90</v>
-      </c>
-      <c r="O6" t="s">
-        <v>91</v>
-      </c>
-      <c r="P6" t="s">
-        <v>92</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>111</v>
-      </c>
-      <c r="R6" t="s">
-        <v>93</v>
-      </c>
-      <c r="S6" t="s">
-        <v>94</v>
-      </c>
-      <c r="T6" t="s">
-        <v>95</v>
-      </c>
-      <c r="U6" t="s">
-        <v>96</v>
-      </c>
-      <c r="V6" t="s">
-        <v>97</v>
-      </c>
-      <c r="W6" t="s">
-        <v>98</v>
-      </c>
-      <c r="X6" t="s">
-        <v>101</v>
-      </c>
-      <c r="Y6" t="s">
-        <v>104</v>
-      </c>
-      <c r="Z6" t="s">
-        <v>99</v>
-      </c>
-      <c r="AA6" t="s">
-        <v>102</v>
-      </c>
-      <c r="AB6" t="s">
-        <v>105</v>
-      </c>
-      <c r="AC6" t="s">
-        <v>100</v>
-      </c>
-      <c r="AD6" t="s">
-        <v>103</v>
-      </c>
-      <c r="AG6" t="s">
-        <v>114</v>
-      </c>
-      <c r="AH6" t="s">
-        <v>108</v>
-      </c>
-      <c r="AI6" t="s">
-        <v>110</v>
-      </c>
-      <c r="AJ6" t="s">
-        <v>109</v>
-      </c>
-      <c r="AK6" t="s">
-        <v>107</v>
-      </c>
-      <c r="AL6" t="s">
-        <v>115</v>
-      </c>
-      <c r="AM6" t="s">
-        <v>116</v>
-      </c>
-      <c r="AN6" t="s">
-        <v>117</v>
-      </c>
-      <c r="AP6" t="s">
-        <v>128</v>
-      </c>
-      <c r="AQ6" t="s">
-        <v>130</v>
-      </c>
-      <c r="AR6" t="s">
-        <v>125</v>
-      </c>
-      <c r="AS6" t="s">
-        <v>132</v>
-      </c>
-      <c r="AT6" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="AU6" t="s">
-        <v>137</v>
-      </c>
-      <c r="AV6" t="s">
-        <v>138</v>
-      </c>
-      <c r="AW6" t="s">
-        <v>139</v>
-      </c>
-      <c r="AX6" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="AY6" t="s">
-        <v>141</v>
-      </c>
-      <c r="AZ6" t="s">
-        <v>142</v>
-      </c>
-      <c r="BA6" t="s">
-        <v>143</v>
-      </c>
-      <c r="BB6" t="s">
-        <v>144</v>
-      </c>
-      <c r="BC6" t="s">
-        <v>145</v>
-      </c>
-      <c r="BD6" t="s">
-        <v>146</v>
-      </c>
-      <c r="BE6" t="s">
-        <v>147</v>
-      </c>
-      <c r="BF6" t="s">
-        <v>148</v>
-      </c>
-      <c r="BG6" t="s">
-        <v>149</v>
-      </c>
-      <c r="BH6" t="s">
-        <v>131</v>
-      </c>
-      <c r="BI6" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="7" spans="1:61" x14ac:dyDescent="0.3">
-      <c r="AG7" t="s">
-        <v>106</v>
-      </c>
-      <c r="AH7" t="s">
-        <v>122</v>
-      </c>
-      <c r="AL7" t="s">
-        <v>113</v>
-      </c>
-      <c r="AP7" t="s">
-        <v>129</v>
-      </c>
-      <c r="AQ7" t="s">
-        <v>131</v>
-      </c>
-      <c r="AR7" t="s">
-        <v>126</v>
-      </c>
-      <c r="AS7" t="s">
-        <v>133</v>
-      </c>
-      <c r="AT7" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="AV7" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="11" spans="1:61" x14ac:dyDescent="0.3">
-      <c r="H11" t="s">
-        <v>120</v>
-      </c>
-      <c r="AO11" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="12" spans="1:61" x14ac:dyDescent="0.3">
-      <c r="H12" t="s">
-        <v>121</v>
-      </c>
-      <c r="AO12" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="13" spans="1:61" x14ac:dyDescent="0.3">
-      <c r="G13" s="6"/>
+      <c r="BG5">
+        <f>IF(MOD(ROW()-5,3) =0,SUM(BA5:BF5),"")</f>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="59">

</xml_diff>